<commit_message>
Add login test scenarios
</commit_message>
<xml_diff>
--- a/Ecom-Test-Scenario.xlsx
+++ b/Ecom-Test-Scenario.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\TS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{57597111-2AC7-4B23-B651-1213ACD55381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4295842C-C639-419D-8B54-5054ECBDF2DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{A1E325CF-020A-4C6B-ADD3-AE6E6645B65D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{A1E325CF-020A-4C6B-ADD3-AE6E6645B65D}"/>
   </bookViews>
   <sheets>
     <sheet name="Home-Page" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="116">
   <si>
     <t>Project Name</t>
   </si>
@@ -68,9 +69,6 @@
     <t>Module</t>
   </si>
   <si>
-    <t>Home Page</t>
-  </si>
-  <si>
     <t>Scenario ID</t>
   </si>
   <si>
@@ -237,6 +235,159 @@
   </si>
   <si>
     <t>Verify that the page URL is correct after the home page loads.</t>
+  </si>
+  <si>
+    <t>Verify that the user can open the Sign In page from the Home Page.</t>
+  </si>
+  <si>
+    <t>Verify that the Sign In page is displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify login with a valid email address and valid password.</t>
+  </si>
+  <si>
+    <t>Verify login with a valid mobile number and valid password.</t>
+  </si>
+  <si>
+    <t>Verify login with an invalid email address.</t>
+  </si>
+  <si>
+    <t>Verify login with an invalid mobile number.</t>
+  </si>
+  <si>
+    <t>Verify login with a valid email address and an incorrect password.</t>
+  </si>
+  <si>
+    <t>Verify login with an empty password field.</t>
+  </si>
+  <si>
+    <t>Verify the validation message for an invalid email or mobile number.</t>
+  </si>
+  <si>
+    <t>Verify the validation message for an incorrect password.</t>
+  </si>
+  <si>
+    <t>Verify the "Forgot Password" functionality.</t>
+  </si>
+  <si>
+    <t>Verify that the "Create your Amazon account" option is available.</t>
+  </si>
+  <si>
+    <t>Verify navigation to the registration page from the Sign In page.</t>
+  </si>
+  <si>
+    <t>Verify that the password is masked while typing.</t>
+  </si>
+  <si>
+    <t>Verify the Show/Hide Password option, if available.</t>
+  </si>
+  <si>
+    <t>Verify the "Keep me signed in" option, if available.</t>
+  </si>
+  <si>
+    <t>Verify login after resetting the password successfully.</t>
+  </si>
+  <si>
+    <t>Verify that the user is redirected to the previous page after a successful login.</t>
+  </si>
+  <si>
+    <t>Verify that the user cannot access the account without successful authentication.</t>
+  </si>
+  <si>
+    <t>Verify that special characters are handled correctly in the login fields.</t>
+  </si>
+  <si>
+    <t>Verify the maximum and minimum input length for the email/mobile field.</t>
+  </si>
+  <si>
+    <t>Verify the maximum password length accepted by the application.</t>
+  </si>
+  <si>
+    <t>Verify that the user can log out successfully after logging in.</t>
+  </si>
+  <si>
+    <t>Login Page</t>
+  </si>
+  <si>
+    <t>TS_Login_001</t>
+  </si>
+  <si>
+    <t>TS_Login_002</t>
+  </si>
+  <si>
+    <t>TS_Login_003</t>
+  </si>
+  <si>
+    <t>TS_Login_004</t>
+  </si>
+  <si>
+    <t>TS_Login_005</t>
+  </si>
+  <si>
+    <t>TS_Login_006</t>
+  </si>
+  <si>
+    <t>TS_Login_007</t>
+  </si>
+  <si>
+    <t>TS_Login_008</t>
+  </si>
+  <si>
+    <t>TS_Login_009</t>
+  </si>
+  <si>
+    <t>TS_Login_010</t>
+  </si>
+  <si>
+    <t>TS_Login_011</t>
+  </si>
+  <si>
+    <t>TS_Login_012</t>
+  </si>
+  <si>
+    <t>TS_Login_013</t>
+  </si>
+  <si>
+    <t>TS_Login_014</t>
+  </si>
+  <si>
+    <t>TS_Login_015</t>
+  </si>
+  <si>
+    <t>TS_Login_016</t>
+  </si>
+  <si>
+    <t>TS_Login_017</t>
+  </si>
+  <si>
+    <t>TS_Login_018</t>
+  </si>
+  <si>
+    <t>TS_Login_019</t>
+  </si>
+  <si>
+    <t>TS_Login_020</t>
+  </si>
+  <si>
+    <t>TS_Login_021</t>
+  </si>
+  <si>
+    <t>TS_Login_022</t>
+  </si>
+  <si>
+    <t>TS_Login_023</t>
+  </si>
+  <si>
+    <t>TS_Login_024</t>
+  </si>
+  <si>
+    <t>TS_Login_025</t>
+  </si>
+  <si>
+    <t>Verify login with an empty email &amp; mobile field.</t>
+  </si>
+  <si>
+    <t>Verify login when both email &amp; mobile and password fields are empty.</t>
   </si>
 </sst>
 </file>
@@ -658,12 +809,312 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C52C776-4B55-4DBE-A115-E873105074AB}">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A9:C34"/>
   <sheetFormatPr defaultColWidth="20.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{580ED6B1-FAC8-4B10-8952-8DCCCC60A8A0}">
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="57.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
@@ -689,7 +1140,7 @@
         <v>8</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>9</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -713,293 +1164,293 @@
         <v>7</v>
       </c>
       <c r="B7" s="5">
-        <v>46212</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>13</v>
+      <c r="A10" s="2" t="s">
+        <v>89</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>15</v>
+        <v>65</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>16</v>
+      <c r="A11" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>15</v>
+        <v>66</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>18</v>
+      <c r="A12" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>20</v>
+        <v>67</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>21</v>
+      <c r="A13" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>15</v>
+        <v>68</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>23</v>
+      <c r="A14" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>15</v>
+        <v>69</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>25</v>
+      <c r="A15" s="2" t="s">
+        <v>94</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>27</v>
+        <v>70</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>95</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>29</v>
+        <v>71</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>96</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>20</v>
+        <v>114</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>31</v>
+      <c r="A18" s="2" t="s">
+        <v>97</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>60</v>
+    </row>
+    <row r="32" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>111</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>62</v>
+        <v>85</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>112</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>33</v>
+        <v>86</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>64</v>
+      <c r="A34" s="2" t="s">
+        <v>113</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>33</v>
+        <v>87</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>